<commit_message>
commit after add new dms
</commit_message>
<xml_diff>
--- a/Master_Document/BUYOFF_Form.xlsx
+++ b/Master_Document/BUYOFF_Form.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.0.5\Users\Acer\IPQC_Project\FamaxQCSystem\Master_Document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{744F9988-148F-4E51-B1C9-B24FE26A5734}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B7B3E0A-742C-46C1-90AE-C98409E47879}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="71">
   <si>
     <r>
       <rPr>
@@ -335,6 +335,9 @@
   </si>
   <si>
     <t>REMARKS (IF ANY)</t>
+  </si>
+  <si>
+    <t>Job Order No:</t>
   </si>
 </sst>
 </file>
@@ -432,86 +435,9 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="38">
+  <borders count="16">
     <border>
       <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
       <right/>
       <top/>
       <bottom/>
@@ -536,15 +462,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -554,17 +471,6 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -603,33 +509,9 @@
     </border>
     <border>
       <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -694,17 +576,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -715,45 +586,6 @@
         <color indexed="64"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -770,56 +602,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -830,553 +612,499 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="20" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
       <protection hidden="1"/>
     </xf>
   </cellXfs>
@@ -1844,823 +1572,854 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="91" t="e" vm="1">
+      <c r="A1" s="99" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="B1" s="92"/>
-      <c r="C1" s="97" t="s">
+      <c r="B1" s="100"/>
+      <c r="C1" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="97"/>
-      <c r="E1" s="97"/>
-      <c r="F1" s="97"/>
-      <c r="G1" s="97"/>
-      <c r="H1" s="97"/>
-      <c r="I1" s="97"/>
-      <c r="J1" s="97"/>
-      <c r="K1" s="81" t="s">
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="65"/>
+      <c r="H1" s="65"/>
+      <c r="I1" s="65"/>
+      <c r="J1" s="65"/>
+      <c r="K1" s="101" t="s">
         <v>1</v>
       </c>
-      <c r="L1" s="50"/>
-      <c r="M1" s="50"/>
-      <c r="N1" s="50"/>
-      <c r="O1" s="50"/>
-      <c r="P1" s="50"/>
-      <c r="Q1" s="50"/>
-      <c r="R1" s="128"/>
-      <c r="S1" s="50" t="e" vm="2">
+      <c r="L1" s="102"/>
+      <c r="M1" s="102"/>
+      <c r="N1" s="102"/>
+      <c r="O1" s="102"/>
+      <c r="P1" s="102"/>
+      <c r="Q1" s="102"/>
+      <c r="R1" s="103"/>
+      <c r="S1" s="102" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="T1" s="50"/>
-      <c r="U1" s="51"/>
+      <c r="T1" s="102"/>
+      <c r="U1" s="103"/>
     </row>
     <row r="2" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="93"/>
-      <c r="B2" s="94"/>
-      <c r="C2" s="98"/>
-      <c r="D2" s="98"/>
-      <c r="E2" s="98"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="98"/>
-      <c r="H2" s="98"/>
-      <c r="I2" s="98"/>
-      <c r="J2" s="98"/>
-      <c r="K2" s="82"/>
-      <c r="L2" s="52"/>
-      <c r="M2" s="52"/>
-      <c r="N2" s="52"/>
-      <c r="O2" s="52"/>
-      <c r="P2" s="52"/>
-      <c r="Q2" s="52"/>
-      <c r="R2" s="129"/>
-      <c r="S2" s="52"/>
-      <c r="T2" s="52"/>
-      <c r="U2" s="53"/>
-    </row>
-    <row r="3" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="95"/>
-      <c r="B3" s="96"/>
-      <c r="C3" s="98"/>
-      <c r="D3" s="98"/>
-      <c r="E3" s="98"/>
-      <c r="F3" s="98"/>
-      <c r="G3" s="98"/>
-      <c r="H3" s="98"/>
-      <c r="I3" s="98"/>
-      <c r="J3" s="98"/>
-      <c r="K3" s="83"/>
+      <c r="A2" s="104"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="65"/>
+      <c r="F2" s="65"/>
+      <c r="G2" s="65"/>
+      <c r="H2" s="65"/>
+      <c r="I2" s="65"/>
+      <c r="J2" s="65"/>
+      <c r="K2" s="51"/>
+      <c r="L2" s="105"/>
+      <c r="M2" s="105"/>
+      <c r="N2" s="105"/>
+      <c r="O2" s="105"/>
+      <c r="P2" s="105"/>
+      <c r="Q2" s="105"/>
+      <c r="R2" s="52"/>
+      <c r="S2" s="105"/>
+      <c r="T2" s="105"/>
+      <c r="U2" s="52"/>
+    </row>
+    <row r="3" spans="1:21" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="106"/>
+      <c r="B3" s="64"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="65"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="65"/>
+      <c r="G3" s="65"/>
+      <c r="H3" s="65"/>
+      <c r="I3" s="65"/>
+      <c r="J3" s="65"/>
+      <c r="K3" s="53"/>
       <c r="L3" s="54"/>
       <c r="M3" s="54"/>
       <c r="N3" s="54"/>
       <c r="O3" s="54"/>
       <c r="P3" s="54"/>
       <c r="Q3" s="54"/>
-      <c r="R3" s="130"/>
-      <c r="S3" s="52"/>
-      <c r="T3" s="52"/>
-      <c r="U3" s="53"/>
+      <c r="R3" s="55"/>
+      <c r="S3" s="105"/>
+      <c r="T3" s="105"/>
+      <c r="U3" s="52"/>
     </row>
     <row r="4" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="73" t="s">
+      <c r="A4" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="39"/>
-      <c r="C4" s="58"/>
-      <c r="D4" s="58"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="58"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="38" t="s">
+      <c r="B4" s="31"/>
+      <c r="C4" s="66"/>
+      <c r="D4" s="66"/>
+      <c r="E4" s="66"/>
+      <c r="F4" s="66"/>
+      <c r="G4" s="66"/>
+      <c r="H4" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="74"/>
-      <c r="J4" s="39"/>
-      <c r="K4" s="38" t="s">
+      <c r="I4" s="38"/>
+      <c r="J4" s="31"/>
+      <c r="K4" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="L4" s="74"/>
-      <c r="M4" s="39"/>
-      <c r="N4" s="38" t="s">
+      <c r="L4" s="38"/>
+      <c r="M4" s="31"/>
+      <c r="N4" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="O4" s="74"/>
-      <c r="P4" s="39"/>
-      <c r="Q4" s="40" t="s">
+      <c r="O4" s="38"/>
+      <c r="P4" s="31"/>
+      <c r="Q4" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="R4" s="42"/>
-      <c r="S4" s="40"/>
-      <c r="T4" s="42"/>
-      <c r="U4" s="125"/>
+      <c r="R4" s="27"/>
+      <c r="S4" s="26"/>
+      <c r="T4" s="27"/>
+      <c r="U4" s="107"/>
     </row>
     <row r="5" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="73" t="s">
+      <c r="A5" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="39"/>
-      <c r="C5" s="58"/>
-      <c r="D5" s="58"/>
-      <c r="E5" s="58"/>
-      <c r="F5" s="58"/>
-      <c r="G5" s="58"/>
-      <c r="H5" s="38" t="s">
+      <c r="B5" s="31"/>
+      <c r="C5" s="66"/>
+      <c r="D5" s="66"/>
+      <c r="E5" s="66"/>
+      <c r="F5" s="66"/>
+      <c r="G5" s="66"/>
+      <c r="H5" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="I5" s="74"/>
-      <c r="J5" s="39"/>
-      <c r="K5" s="38" t="s">
+      <c r="I5" s="38"/>
+      <c r="J5" s="31"/>
+      <c r="K5" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="L5" s="74"/>
-      <c r="M5" s="39"/>
-      <c r="N5" s="38" t="s">
+      <c r="L5" s="38"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="O5" s="74"/>
-      <c r="P5" s="39"/>
-      <c r="Q5" s="41"/>
-      <c r="R5" s="43"/>
-      <c r="S5" s="41"/>
-      <c r="T5" s="43"/>
-      <c r="U5" s="78"/>
+      <c r="O5" s="38"/>
+      <c r="P5" s="31"/>
+      <c r="Q5" s="28"/>
+      <c r="R5" s="29"/>
+      <c r="S5" s="28"/>
+      <c r="T5" s="29"/>
+      <c r="U5" s="108"/>
     </row>
     <row r="6" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="73" t="s">
+      <c r="A6" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="39"/>
-      <c r="C6" s="58"/>
-      <c r="D6" s="58"/>
-      <c r="E6" s="58"/>
-      <c r="F6" s="58"/>
-      <c r="G6" s="58"/>
-      <c r="H6" s="59"/>
-      <c r="I6" s="60"/>
-      <c r="J6" s="61"/>
-      <c r="K6" s="59"/>
-      <c r="L6" s="60"/>
-      <c r="M6" s="61"/>
-      <c r="N6" s="59"/>
-      <c r="O6" s="60"/>
-      <c r="P6" s="61"/>
-      <c r="Q6" s="38" t="s">
+      <c r="B6" s="31"/>
+      <c r="C6" s="66"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
+      <c r="G6" s="66"/>
+      <c r="H6" s="67"/>
+      <c r="I6" s="68"/>
+      <c r="J6" s="69"/>
+      <c r="K6" s="67"/>
+      <c r="L6" s="68"/>
+      <c r="M6" s="69"/>
+      <c r="N6" s="67"/>
+      <c r="O6" s="68"/>
+      <c r="P6" s="69"/>
+      <c r="Q6" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="R6" s="39"/>
-      <c r="S6" s="41"/>
-      <c r="T6" s="43"/>
-      <c r="U6" s="78"/>
+      <c r="R6" s="31"/>
+      <c r="S6" s="28"/>
+      <c r="T6" s="29"/>
+      <c r="U6" s="108"/>
     </row>
     <row r="7" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="73" t="s">
+      <c r="A7" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="39"/>
-      <c r="C7" s="58"/>
-      <c r="D7" s="58"/>
-      <c r="E7" s="58"/>
-      <c r="F7" s="58"/>
-      <c r="G7" s="58"/>
-      <c r="H7" s="62"/>
-      <c r="I7" s="63"/>
-      <c r="J7" s="64"/>
-      <c r="K7" s="62"/>
-      <c r="L7" s="63"/>
-      <c r="M7" s="64"/>
-      <c r="N7" s="62"/>
-      <c r="O7" s="63"/>
-      <c r="P7" s="64"/>
-      <c r="Q7" s="38" t="s">
+      <c r="B7" s="31"/>
+      <c r="C7" s="66"/>
+      <c r="D7" s="66"/>
+      <c r="E7" s="66"/>
+      <c r="F7" s="66"/>
+      <c r="G7" s="66"/>
+      <c r="H7" s="70"/>
+      <c r="I7" s="109"/>
+      <c r="J7" s="71"/>
+      <c r="K7" s="70"/>
+      <c r="L7" s="109"/>
+      <c r="M7" s="71"/>
+      <c r="N7" s="70"/>
+      <c r="O7" s="109"/>
+      <c r="P7" s="71"/>
+      <c r="Q7" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="R7" s="39"/>
-      <c r="S7" s="55" t="str">
+      <c r="R7" s="31"/>
+      <c r="S7" s="56" t="str">
         <f>IF(O9&lt;&gt;"", O9+7, "")</f>
         <v/>
       </c>
-      <c r="T7" s="56"/>
-      <c r="U7" s="57"/>
+      <c r="T7" s="57"/>
+      <c r="U7" s="110"/>
     </row>
     <row r="8" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="73" t="s">
+      <c r="A8" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="39"/>
-      <c r="C8" s="58"/>
-      <c r="D8" s="58"/>
-      <c r="E8" s="58"/>
-      <c r="F8" s="58"/>
-      <c r="G8" s="58"/>
-      <c r="H8" s="65"/>
-      <c r="I8" s="63"/>
-      <c r="J8" s="67"/>
-      <c r="K8" s="65"/>
-      <c r="L8" s="66"/>
-      <c r="M8" s="67"/>
-      <c r="N8" s="65"/>
-      <c r="O8" s="66"/>
-      <c r="P8" s="67"/>
-      <c r="Q8" s="38" t="s">
+      <c r="B8" s="31"/>
+      <c r="C8" s="66"/>
+      <c r="D8" s="66"/>
+      <c r="E8" s="66"/>
+      <c r="F8" s="66"/>
+      <c r="G8" s="66"/>
+      <c r="H8" s="72"/>
+      <c r="I8" s="109"/>
+      <c r="J8" s="73"/>
+      <c r="K8" s="72"/>
+      <c r="L8" s="74"/>
+      <c r="M8" s="73"/>
+      <c r="N8" s="72"/>
+      <c r="O8" s="74"/>
+      <c r="P8" s="73"/>
+      <c r="Q8" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="R8" s="39"/>
-      <c r="S8" s="21">
+      <c r="R8" s="31"/>
+      <c r="S8" s="12">
         <v>1</v>
       </c>
-      <c r="T8" s="21" t="s">
+      <c r="T8" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="U8" s="24">
+      <c r="U8" s="12">
         <f>COUNTA(A15,#REF!,#REF!,#REF!,#REF!,#REF!,#REF!,#REF!,#REF!,#REF!)</f>
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="73" t="s">
+      <c r="A9" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="39"/>
-      <c r="C9" s="38"/>
-      <c r="D9" s="74"/>
-      <c r="E9" s="39"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="37" t="s">
+      <c r="B9" s="31"/>
+      <c r="C9" s="30"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="31"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="I9" s="69"/>
-      <c r="J9" s="70"/>
-      <c r="K9" s="37" t="s">
+      <c r="I9" s="75"/>
+      <c r="J9" s="58"/>
+      <c r="K9" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="L9" s="70"/>
-      <c r="M9" s="70"/>
-      <c r="N9" s="37" t="s">
+      <c r="L9" s="58"/>
+      <c r="M9" s="58"/>
+      <c r="N9" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="O9" s="71"/>
-      <c r="P9" s="72"/>
-      <c r="Q9" s="27"/>
-      <c r="R9" s="27"/>
-      <c r="S9" s="27"/>
-      <c r="T9" s="27"/>
-      <c r="U9" s="28"/>
+      <c r="O9" s="32"/>
+      <c r="P9" s="33"/>
+      <c r="Q9" s="111"/>
+      <c r="R9" s="111"/>
+      <c r="S9" s="111"/>
+      <c r="T9" s="111"/>
+      <c r="U9" s="112"/>
     </row>
     <row r="10" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="73" t="s">
+      <c r="A10" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="39"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21" t="s">
+      <c r="B10" s="31"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="E10" s="21"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="84" t="s">
+      <c r="E10" s="12"/>
+      <c r="F10" s="111"/>
+      <c r="G10" s="76" t="s">
         <v>31</v>
       </c>
-      <c r="H10" s="29" t="s">
+      <c r="H10" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="I10" s="119"/>
-      <c r="J10" s="120"/>
-      <c r="K10" s="26" t="s">
+      <c r="I10" s="77"/>
+      <c r="J10" s="78"/>
+      <c r="K10" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="L10" s="30"/>
-      <c r="M10" s="27"/>
-      <c r="N10" s="68" t="s">
+      <c r="L10" s="18"/>
+      <c r="M10" s="111"/>
+      <c r="N10" s="79" t="s">
         <v>34</v>
       </c>
-      <c r="O10" s="21" t="s">
+      <c r="O10" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="P10" s="23"/>
-      <c r="Q10" s="27"/>
-      <c r="R10" s="27"/>
-      <c r="S10" s="27"/>
-      <c r="T10" s="27"/>
-      <c r="U10" s="28"/>
+      <c r="P10" s="14"/>
+      <c r="Q10" s="49" t="s">
+        <v>70</v>
+      </c>
+      <c r="R10" s="113"/>
+      <c r="S10" s="113"/>
+      <c r="T10" s="113"/>
+      <c r="U10" s="114"/>
     </row>
     <row r="11" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="31"/>
-      <c r="B11" s="27"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="84"/>
-      <c r="H11" s="29" t="s">
+      <c r="A11" s="25"/>
+      <c r="B11" s="111"/>
+      <c r="C11" s="111"/>
+      <c r="D11" s="111"/>
+      <c r="E11" s="111"/>
+      <c r="F11" s="111"/>
+      <c r="G11" s="76"/>
+      <c r="H11" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="I11" s="89"/>
-      <c r="J11" s="90"/>
-      <c r="K11" s="32" t="s">
+      <c r="I11" s="45"/>
+      <c r="J11" s="46"/>
+      <c r="K11" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="L11" s="30"/>
-      <c r="M11" s="27"/>
-      <c r="N11" s="68"/>
-      <c r="O11" s="21" t="s">
+      <c r="L11" s="18"/>
+      <c r="M11" s="111"/>
+      <c r="N11" s="79"/>
+      <c r="O11" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="P11" s="30"/>
-      <c r="Q11" s="85" t="s">
+      <c r="P11" s="18"/>
+      <c r="Q11" s="59" t="s">
         <v>44</v>
       </c>
-      <c r="R11" s="86"/>
-      <c r="S11" s="23"/>
-      <c r="T11" s="27"/>
-      <c r="U11" s="28"/>
+      <c r="R11" s="60"/>
+      <c r="S11" s="50"/>
+      <c r="T11" s="115"/>
+      <c r="U11" s="116"/>
     </row>
     <row r="12" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="5"/>
-      <c r="U12" s="4"/>
+      <c r="A12" s="117"/>
+      <c r="B12" s="118"/>
+      <c r="C12" s="118"/>
+      <c r="D12" s="118"/>
+      <c r="E12" s="118"/>
+      <c r="F12" s="118"/>
+      <c r="G12" s="118"/>
+      <c r="H12" s="118"/>
+      <c r="I12" s="118"/>
+      <c r="J12" s="118"/>
+      <c r="K12" s="118"/>
+      <c r="L12" s="118"/>
+      <c r="M12" s="118"/>
+      <c r="N12" s="118"/>
+      <c r="O12" s="118"/>
+      <c r="P12" s="118"/>
+      <c r="Q12" s="118"/>
+      <c r="R12" s="118"/>
+      <c r="S12" s="118"/>
+      <c r="T12" s="118"/>
+      <c r="U12" s="119"/>
     </row>
     <row r="13" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="126" t="s">
+      <c r="A13" s="85" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="68" t="s">
+      <c r="B13" s="79" t="s">
         <v>45</v>
       </c>
-      <c r="C13" s="68"/>
-      <c r="D13" s="20" t="s">
+      <c r="C13" s="79"/>
+      <c r="D13" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="21" t="s">
+      <c r="E13" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="F13" s="21" t="s">
+      <c r="F13" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="G13" s="38" t="s">
+      <c r="G13" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="H13" s="39"/>
-      <c r="I13" s="121" t="s">
+      <c r="H13" s="31"/>
+      <c r="I13" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="J13" s="122"/>
-      <c r="K13" s="38" t="s">
+      <c r="J13" s="35"/>
+      <c r="K13" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="L13" s="74"/>
-      <c r="M13" s="74"/>
-      <c r="N13" s="74"/>
-      <c r="O13" s="39"/>
-      <c r="P13" s="38" t="s">
+      <c r="L13" s="38"/>
+      <c r="M13" s="38"/>
+      <c r="N13" s="38"/>
+      <c r="O13" s="31"/>
+      <c r="P13" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="Q13" s="74"/>
-      <c r="R13" s="74"/>
-      <c r="S13" s="74"/>
-      <c r="T13" s="39"/>
-      <c r="U13" s="4"/>
+      <c r="Q13" s="38"/>
+      <c r="R13" s="38"/>
+      <c r="S13" s="38"/>
+      <c r="T13" s="31"/>
+      <c r="U13" s="119"/>
     </row>
     <row r="14" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="127"/>
-      <c r="B14" s="68"/>
-      <c r="C14" s="68"/>
-      <c r="D14" s="20" t="s">
+      <c r="A14" s="87"/>
+      <c r="B14" s="79"/>
+      <c r="C14" s="79"/>
+      <c r="D14" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="E14" s="21" t="s">
+      <c r="E14" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="F14" s="21" t="s">
+      <c r="F14" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G14" s="21" t="s">
+      <c r="G14" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="H14" s="21" t="s">
+      <c r="H14" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="I14" s="123"/>
-      <c r="J14" s="124"/>
-      <c r="K14" s="21">
+      <c r="I14" s="36"/>
+      <c r="J14" s="37"/>
+      <c r="K14" s="12">
         <v>1</v>
       </c>
-      <c r="L14" s="21">
+      <c r="L14" s="12">
         <v>2</v>
       </c>
-      <c r="M14" s="21">
+      <c r="M14" s="12">
         <v>3</v>
       </c>
-      <c r="N14" s="21">
+      <c r="N14" s="12">
         <v>4</v>
       </c>
-      <c r="O14" s="21">
+      <c r="O14" s="12">
         <v>5</v>
       </c>
-      <c r="P14" s="21">
+      <c r="P14" s="12">
         <v>1</v>
       </c>
-      <c r="Q14" s="21">
+      <c r="Q14" s="12">
         <v>2</v>
       </c>
-      <c r="R14" s="21">
+      <c r="R14" s="12">
         <v>3</v>
       </c>
-      <c r="S14" s="21">
+      <c r="S14" s="12">
         <v>4</v>
       </c>
-      <c r="T14" s="21">
+      <c r="T14" s="12">
         <v>5</v>
       </c>
-      <c r="U14" s="4"/>
+      <c r="U14" s="119"/>
     </row>
     <row r="15" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="33"/>
-      <c r="B15" s="101"/>
-      <c r="C15" s="102"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="35"/>
-      <c r="F15" s="35" t="s">
+      <c r="A15" s="24"/>
+      <c r="B15" s="80"/>
+      <c r="C15" s="81"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="G15" s="35" t="str">
+      <c r="G15" s="21" t="str">
         <f t="shared" ref="G15:G26" si="0">IF(ISNUMBER(D15),(D15+E15)/2-3*(E15 - (D15+E15)/2) / (3 * F29),"")</f>
         <v/>
       </c>
-      <c r="H15" s="35" t="str">
+      <c r="H15" s="21" t="str">
         <f t="shared" ref="H15:H26" si="1">IF(ISNUMBER(E15),(D15+E15)/2+3*(E15 - (D15+E15)/2) / (3 * F29),"")</f>
         <v/>
       </c>
-      <c r="I15" s="99"/>
-      <c r="J15" s="100"/>
-      <c r="K15" s="36"/>
-      <c r="L15" s="36"/>
-      <c r="M15" s="36"/>
-      <c r="N15" s="36"/>
-      <c r="O15" s="36"/>
-      <c r="P15" s="36"/>
-      <c r="Q15" s="36"/>
-      <c r="R15" s="36"/>
-      <c r="S15" s="36"/>
-      <c r="T15" s="36"/>
-      <c r="U15" s="4"/>
+      <c r="I15" s="47"/>
+      <c r="J15" s="48"/>
+      <c r="K15" s="22"/>
+      <c r="L15" s="22"/>
+      <c r="M15" s="22"/>
+      <c r="N15" s="22"/>
+      <c r="O15" s="22"/>
+      <c r="P15" s="22"/>
+      <c r="Q15" s="22"/>
+      <c r="R15" s="22"/>
+      <c r="S15" s="22"/>
+      <c r="T15" s="22"/>
+      <c r="U15" s="119"/>
     </row>
     <row r="16" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="33"/>
-      <c r="B16" s="101"/>
-      <c r="C16" s="102"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="35"/>
-      <c r="F16" s="35" t="s">
+      <c r="A16" s="24"/>
+      <c r="B16" s="80"/>
+      <c r="C16" s="81"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="G16" s="35" t="str">
+      <c r="G16" s="21" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H16" s="35" t="str">
+      <c r="H16" s="21" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="I16" s="99"/>
-      <c r="J16" s="100"/>
-      <c r="K16" s="36"/>
-      <c r="L16" s="36"/>
-      <c r="M16" s="36"/>
-      <c r="N16" s="36"/>
-      <c r="O16" s="36"/>
-      <c r="P16" s="36"/>
-      <c r="Q16" s="36"/>
-      <c r="R16" s="36"/>
-      <c r="S16" s="36"/>
-      <c r="T16" s="36"/>
-      <c r="U16" s="4"/>
+      <c r="I16" s="47"/>
+      <c r="J16" s="48"/>
+      <c r="K16" s="22"/>
+      <c r="L16" s="22"/>
+      <c r="M16" s="22"/>
+      <c r="N16" s="22"/>
+      <c r="O16" s="22"/>
+      <c r="P16" s="22"/>
+      <c r="Q16" s="22"/>
+      <c r="R16" s="22"/>
+      <c r="S16" s="22"/>
+      <c r="T16" s="22"/>
+      <c r="U16" s="119"/>
     </row>
     <row r="17" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="33"/>
-      <c r="B17" s="101"/>
-      <c r="C17" s="102"/>
-      <c r="D17" s="34"/>
-      <c r="E17" s="35"/>
-      <c r="F17" s="35" t="s">
+      <c r="A17" s="24"/>
+      <c r="B17" s="80"/>
+      <c r="C17" s="81"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="G17" s="35" t="str">
+      <c r="G17" s="21" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H17" s="35" t="str">
+      <c r="H17" s="21" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="I17" s="99"/>
-      <c r="J17" s="100"/>
-      <c r="K17" s="36"/>
-      <c r="L17" s="36"/>
-      <c r="M17" s="36"/>
-      <c r="N17" s="36"/>
-      <c r="O17" s="36"/>
-      <c r="P17" s="36"/>
-      <c r="Q17" s="36"/>
-      <c r="R17" s="36"/>
-      <c r="S17" s="36"/>
-      <c r="T17" s="36"/>
-      <c r="U17" s="4"/>
+      <c r="I17" s="47"/>
+      <c r="J17" s="48"/>
+      <c r="K17" s="22"/>
+      <c r="L17" s="22"/>
+      <c r="M17" s="22"/>
+      <c r="N17" s="22"/>
+      <c r="O17" s="22"/>
+      <c r="P17" s="22"/>
+      <c r="Q17" s="22"/>
+      <c r="R17" s="22"/>
+      <c r="S17" s="22"/>
+      <c r="T17" s="22"/>
+      <c r="U17" s="119"/>
     </row>
     <row r="18" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="33"/>
-      <c r="B18" s="101"/>
-      <c r="C18" s="102"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="35"/>
-      <c r="F18" s="35" t="s">
+      <c r="A18" s="24"/>
+      <c r="B18" s="80"/>
+      <c r="C18" s="81"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="G18" s="35" t="str">
+      <c r="G18" s="21" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H18" s="35" t="str">
+      <c r="H18" s="21" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="I18" s="99"/>
-      <c r="J18" s="100"/>
-      <c r="K18" s="36"/>
-      <c r="L18" s="36"/>
-      <c r="M18" s="36"/>
-      <c r="N18" s="36"/>
-      <c r="O18" s="36"/>
-      <c r="P18" s="36"/>
-      <c r="Q18" s="36"/>
-      <c r="R18" s="36"/>
-      <c r="S18" s="36"/>
-      <c r="T18" s="36"/>
-      <c r="U18" s="4"/>
+      <c r="I18" s="47"/>
+      <c r="J18" s="48"/>
+      <c r="K18" s="22"/>
+      <c r="L18" s="22"/>
+      <c r="M18" s="22"/>
+      <c r="N18" s="22"/>
+      <c r="O18" s="22"/>
+      <c r="P18" s="22"/>
+      <c r="Q18" s="22"/>
+      <c r="R18" s="22"/>
+      <c r="S18" s="22"/>
+      <c r="T18" s="22"/>
+      <c r="U18" s="119"/>
     </row>
     <row r="19" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="33"/>
-      <c r="B19" s="101"/>
-      <c r="C19" s="102"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="35"/>
-      <c r="F19" s="35" t="s">
+      <c r="A19" s="24"/>
+      <c r="B19" s="80"/>
+      <c r="C19" s="81"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="G19" s="35" t="str">
+      <c r="G19" s="21" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H19" s="35" t="str">
+      <c r="H19" s="21" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="I19" s="99"/>
-      <c r="J19" s="100"/>
-      <c r="K19" s="36"/>
-      <c r="L19" s="36"/>
-      <c r="M19" s="36"/>
-      <c r="N19" s="36"/>
-      <c r="O19" s="36"/>
-      <c r="P19" s="36"/>
-      <c r="Q19" s="36"/>
-      <c r="R19" s="36"/>
-      <c r="S19" s="36"/>
-      <c r="T19" s="36"/>
-      <c r="U19" s="4"/>
+      <c r="I19" s="47"/>
+      <c r="J19" s="48"/>
+      <c r="K19" s="22"/>
+      <c r="L19" s="22"/>
+      <c r="M19" s="22"/>
+      <c r="N19" s="22"/>
+      <c r="O19" s="22"/>
+      <c r="P19" s="22"/>
+      <c r="Q19" s="22"/>
+      <c r="R19" s="22"/>
+      <c r="S19" s="22"/>
+      <c r="T19" s="22"/>
+      <c r="U19" s="119"/>
     </row>
     <row r="20" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="33"/>
-      <c r="B20" s="101"/>
-      <c r="C20" s="102"/>
-      <c r="D20" s="34"/>
-      <c r="E20" s="35"/>
-      <c r="F20" s="35" t="s">
+      <c r="A20" s="24"/>
+      <c r="B20" s="80"/>
+      <c r="C20" s="81"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="G20" s="35" t="str">
+      <c r="G20" s="21" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H20" s="35" t="str">
+      <c r="H20" s="21" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="I20" s="99"/>
-      <c r="J20" s="100"/>
-      <c r="K20" s="36"/>
-      <c r="L20" s="36"/>
-      <c r="M20" s="36"/>
-      <c r="N20" s="36"/>
-      <c r="O20" s="36"/>
-      <c r="P20" s="36"/>
-      <c r="Q20" s="36"/>
-      <c r="R20" s="36"/>
-      <c r="S20" s="36"/>
-      <c r="T20" s="36"/>
-      <c r="U20" s="4"/>
+      <c r="I20" s="47"/>
+      <c r="J20" s="48"/>
+      <c r="K20" s="22"/>
+      <c r="L20" s="22"/>
+      <c r="M20" s="22"/>
+      <c r="N20" s="22"/>
+      <c r="O20" s="22"/>
+      <c r="P20" s="22"/>
+      <c r="Q20" s="22"/>
+      <c r="R20" s="22"/>
+      <c r="S20" s="22"/>
+      <c r="T20" s="22"/>
+      <c r="U20" s="119"/>
     </row>
     <row r="21" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="33"/>
-      <c r="B21" s="101"/>
-      <c r="C21" s="102"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="35"/>
-      <c r="F21" s="35" t="s">
+      <c r="A21" s="24"/>
+      <c r="B21" s="80"/>
+      <c r="C21" s="81"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="21"/>
+      <c r="F21" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="G21" s="35" t="str">
+      <c r="G21" s="21" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H21" s="35" t="str">
+      <c r="H21" s="21" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="I21" s="99"/>
-      <c r="J21" s="100"/>
-      <c r="K21" s="36"/>
-      <c r="L21" s="36"/>
-      <c r="M21" s="36"/>
-      <c r="N21" s="36"/>
-      <c r="O21" s="36"/>
-      <c r="P21" s="36"/>
-      <c r="Q21" s="36"/>
-      <c r="R21" s="36"/>
-      <c r="S21" s="36"/>
-      <c r="T21" s="36"/>
-      <c r="U21" s="4"/>
+      <c r="I21" s="47"/>
+      <c r="J21" s="48"/>
+      <c r="K21" s="22"/>
+      <c r="L21" s="22"/>
+      <c r="M21" s="22"/>
+      <c r="N21" s="22"/>
+      <c r="O21" s="22"/>
+      <c r="P21" s="22"/>
+      <c r="Q21" s="22"/>
+      <c r="R21" s="22"/>
+      <c r="S21" s="22"/>
+      <c r="T21" s="22"/>
+      <c r="U21" s="119"/>
     </row>
     <row r="22" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="33"/>
-      <c r="B22" s="101"/>
-      <c r="C22" s="102"/>
-      <c r="D22" s="34"/>
-      <c r="E22" s="35"/>
-      <c r="F22" s="35" t="s">
+      <c r="A22" s="24"/>
+      <c r="B22" s="80"/>
+      <c r="C22" s="81"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="21"/>
+      <c r="F22" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="G22" s="35" t="str">
+      <c r="G22" s="21" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H22" s="35" t="str">
+      <c r="H22" s="21" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="I22" s="99"/>
-      <c r="J22" s="100"/>
-      <c r="K22" s="36"/>
-      <c r="L22" s="36"/>
-      <c r="M22" s="36"/>
-      <c r="N22" s="36"/>
-      <c r="O22" s="36"/>
-      <c r="P22" s="36"/>
-      <c r="Q22" s="36"/>
-      <c r="R22" s="36"/>
-      <c r="S22" s="36"/>
-      <c r="T22" s="36"/>
-      <c r="U22" s="4"/>
+      <c r="I22" s="47"/>
+      <c r="J22" s="48"/>
+      <c r="K22" s="22"/>
+      <c r="L22" s="22"/>
+      <c r="M22" s="22"/>
+      <c r="N22" s="22"/>
+      <c r="O22" s="22"/>
+      <c r="P22" s="22"/>
+      <c r="Q22" s="22"/>
+      <c r="R22" s="22"/>
+      <c r="S22" s="22"/>
+      <c r="T22" s="22"/>
+      <c r="U22" s="119"/>
     </row>
     <row r="23" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="33"/>
-      <c r="B23" s="101"/>
-      <c r="C23" s="102"/>
-      <c r="D23" s="34"/>
-      <c r="E23" s="35"/>
-      <c r="F23" s="35" t="s">
+      <c r="A23" s="24"/>
+      <c r="B23" s="80"/>
+      <c r="C23" s="81"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="G23" s="35" t="str">
+      <c r="G23" s="21" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H23" s="35" t="str">
+      <c r="H23" s="21" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="I23" s="99"/>
-      <c r="J23" s="100"/>
-      <c r="K23" s="36"/>
-      <c r="L23" s="36"/>
-      <c r="M23" s="36"/>
-      <c r="N23" s="36"/>
-      <c r="O23" s="36"/>
-      <c r="P23" s="36"/>
-      <c r="Q23" s="36"/>
-      <c r="R23" s="36"/>
-      <c r="S23" s="36"/>
-      <c r="T23" s="36"/>
-      <c r="U23" s="4"/>
+      <c r="I23" s="47"/>
+      <c r="J23" s="48"/>
+      <c r="K23" s="22"/>
+      <c r="L23" s="22"/>
+      <c r="M23" s="22"/>
+      <c r="N23" s="22"/>
+      <c r="O23" s="22"/>
+      <c r="P23" s="22"/>
+      <c r="Q23" s="22"/>
+      <c r="R23" s="22"/>
+      <c r="S23" s="22"/>
+      <c r="T23" s="22"/>
+      <c r="U23" s="119"/>
     </row>
     <row r="24" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="33"/>
-      <c r="B24" s="101"/>
-      <c r="C24" s="102"/>
-      <c r="D24" s="34"/>
-      <c r="E24" s="35"/>
-      <c r="F24" s="35" t="s">
+      <c r="A24" s="24"/>
+      <c r="B24" s="80"/>
+      <c r="C24" s="81"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="G24" s="35" t="str">
+      <c r="G24" s="21" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H24" s="35" t="str">
+      <c r="H24" s="21" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="I24" s="99"/>
-      <c r="J24" s="100"/>
-      <c r="K24" s="36"/>
-      <c r="L24" s="36"/>
-      <c r="M24" s="36"/>
-      <c r="N24" s="36"/>
-      <c r="O24" s="36"/>
-      <c r="P24" s="36"/>
-      <c r="Q24" s="36"/>
-      <c r="R24" s="36"/>
-      <c r="S24" s="36"/>
-      <c r="T24" s="36"/>
-      <c r="U24" s="4"/>
+      <c r="I24" s="47"/>
+      <c r="J24" s="48"/>
+      <c r="K24" s="22"/>
+      <c r="L24" s="22"/>
+      <c r="M24" s="22"/>
+      <c r="N24" s="22"/>
+      <c r="O24" s="22"/>
+      <c r="P24" s="22"/>
+      <c r="Q24" s="22"/>
+      <c r="R24" s="22"/>
+      <c r="S24" s="22"/>
+      <c r="T24" s="22"/>
+      <c r="U24" s="119"/>
     </row>
     <row r="25" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="33"/>
-      <c r="B25" s="101"/>
-      <c r="C25" s="102"/>
-      <c r="D25" s="34"/>
-      <c r="E25" s="35"/>
-      <c r="F25" s="35" t="s">
+      <c r="A25" s="24"/>
+      <c r="B25" s="80"/>
+      <c r="C25" s="81"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="G25" s="35" t="str">
+      <c r="G25" s="21" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H25" s="35" t="str">
+      <c r="H25" s="21" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="I25" s="99"/>
-      <c r="J25" s="100"/>
-      <c r="K25" s="36"/>
-      <c r="L25" s="36"/>
-      <c r="M25" s="36"/>
-      <c r="N25" s="36"/>
-      <c r="O25" s="36"/>
-      <c r="P25" s="36"/>
-      <c r="Q25" s="36"/>
-      <c r="R25" s="36"/>
-      <c r="S25" s="36"/>
-      <c r="T25" s="36"/>
-      <c r="U25" s="4"/>
+      <c r="I25" s="47"/>
+      <c r="J25" s="48"/>
+      <c r="K25" s="22"/>
+      <c r="L25" s="22"/>
+      <c r="M25" s="22"/>
+      <c r="N25" s="22"/>
+      <c r="O25" s="22"/>
+      <c r="P25" s="22"/>
+      <c r="Q25" s="22"/>
+      <c r="R25" s="22"/>
+      <c r="S25" s="22"/>
+      <c r="T25" s="22"/>
+      <c r="U25" s="119"/>
     </row>
     <row r="26" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="33"/>
-      <c r="B26" s="101"/>
-      <c r="C26" s="102"/>
-      <c r="D26" s="34"/>
-      <c r="E26" s="35"/>
-      <c r="F26" s="35" t="s">
+      <c r="A26" s="24"/>
+      <c r="B26" s="80"/>
+      <c r="C26" s="81"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="G26" s="35" t="str">
+      <c r="G26" s="21" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="H26" s="35" t="str">
+      <c r="H26" s="21" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="I26" s="99"/>
-      <c r="J26" s="100"/>
-      <c r="K26" s="36"/>
-      <c r="L26" s="36"/>
-      <c r="M26" s="36"/>
-      <c r="N26" s="36"/>
-      <c r="O26" s="36"/>
-      <c r="P26" s="36"/>
-      <c r="Q26" s="36"/>
-      <c r="R26" s="36"/>
-      <c r="S26" s="36"/>
-      <c r="T26" s="36"/>
-      <c r="U26" s="4"/>
+      <c r="I26" s="47"/>
+      <c r="J26" s="48"/>
+      <c r="K26" s="22"/>
+      <c r="L26" s="22"/>
+      <c r="M26" s="22"/>
+      <c r="N26" s="22"/>
+      <c r="O26" s="22"/>
+      <c r="P26" s="22"/>
+      <c r="Q26" s="22"/>
+      <c r="R26" s="22"/>
+      <c r="S26" s="22"/>
+      <c r="T26" s="22"/>
+      <c r="U26" s="119"/>
     </row>
     <row r="27" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="87" t="s">
+      <c r="A27" s="61" t="s">
         <v>47</v>
       </c>
-      <c r="B27" s="88"/>
-      <c r="C27" s="88"/>
-      <c r="D27" s="88"/>
-      <c r="E27" s="88"/>
-      <c r="F27" s="88"/>
-      <c r="G27" s="88"/>
-      <c r="H27" s="88"/>
-      <c r="I27" s="88"/>
-      <c r="J27" s="80"/>
-      <c r="U27" s="4"/>
+      <c r="B27" s="82"/>
+      <c r="C27" s="82"/>
+      <c r="D27" s="82"/>
+      <c r="E27" s="82"/>
+      <c r="F27" s="82"/>
+      <c r="G27" s="82"/>
+      <c r="H27" s="82"/>
+      <c r="I27" s="82"/>
+      <c r="J27" s="62"/>
+      <c r="K27" s="118"/>
+      <c r="L27" s="118"/>
+      <c r="M27" s="118"/>
+      <c r="N27" s="118"/>
+      <c r="O27" s="118"/>
+      <c r="P27" s="118"/>
+      <c r="Q27" s="118"/>
+      <c r="R27" s="118"/>
+      <c r="S27" s="118"/>
+      <c r="T27" s="118"/>
+      <c r="U27" s="119"/>
     </row>
     <row r="28" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="8"/>
+      <c r="A28" s="120"/>
       <c r="B28" s="2" t="s">
         <v>48</v>
       </c>
@@ -2670,7 +2429,7 @@
       <c r="D28" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E28" s="9" t="s">
+      <c r="E28" s="6" t="s">
         <v>51</v>
       </c>
       <c r="F28" s="3" t="s">
@@ -2688,719 +2447,883 @@
       <c r="J28" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="U28" s="4"/>
+      <c r="K28" s="118"/>
+      <c r="L28" s="118"/>
+      <c r="M28" s="118"/>
+      <c r="N28" s="118"/>
+      <c r="O28" s="118"/>
+      <c r="P28" s="118"/>
+      <c r="Q28" s="118"/>
+      <c r="R28" s="118"/>
+      <c r="S28" s="118"/>
+      <c r="T28" s="118"/>
+      <c r="U28" s="119"/>
     </row>
     <row r="29" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="10" t="str">
+      <c r="A29" s="5" t="str">
         <f>IF(ISBLANK(A15),"",A15)</f>
         <v/>
       </c>
-      <c r="B29" s="7" t="str" cm="1">
+      <c r="B29" s="5" t="str" cm="1">
         <f t="array" ref="B29">IF(D15="", "", IF(AND(D15&lt;=MIN(K15:T15),E15&gt;=MAX(K15:T15)),"ACCEPT",IF(AND(K15:T15="OK"),"ACCEPT","REJECT")))</f>
         <v/>
       </c>
-      <c r="C29" s="7" t="str">
+      <c r="C29" s="5" t="str">
         <f t="shared" ref="C29:C40" si="2">IF(TRIM(B29)="", "", MAX(K15:T15))</f>
         <v/>
       </c>
-      <c r="D29" s="7" t="str">
+      <c r="D29" s="5" t="str">
         <f t="shared" ref="D29:D40" si="3">IF(TRIM(B29)="", "", MIN(K15:T15))</f>
         <v/>
       </c>
-      <c r="E29" s="7" t="str">
+      <c r="E29" s="5" t="str">
         <f t="shared" ref="E29:E40" si="4">IF(ISNUMBER(D15),"VARIABLE",IF(ISBLANK(D15),"","ATTRIBUTE"))</f>
         <v/>
       </c>
-      <c r="F29" s="7">
+      <c r="F29" s="5">
         <f t="shared" ref="F29:F40" si="5">IF((F15="QC"),1.33,1)</f>
         <v>1</v>
       </c>
-      <c r="G29" s="7">
+      <c r="G29" s="5">
         <f t="shared" ref="G29:G40" si="6">IF(COUNT(K15:T15)=0,0,AVERAGE(K15:T15))</f>
         <v>0</v>
       </c>
-      <c r="H29" s="7">
+      <c r="H29" s="5">
         <f t="shared" ref="H29:H40" si="7">MAX(K15:T15)-MIN(K15:T15)</f>
         <v>0</v>
       </c>
-      <c r="I29" s="7">
+      <c r="I29" s="5">
         <f t="shared" ref="I29:I40" si="8">IF(COUNT(K15:T15)=0,0,_xlfn.STDEV.S(K15:T15))</f>
         <v>0</v>
       </c>
-      <c r="J29" s="7" t="str">
+      <c r="J29" s="5" t="str">
         <f t="shared" ref="J29:J40" si="9">IF(G29=0,"-",IF(G29-D15&lt;E15-G29,G29-D15,E15-G29)/(I29*3))</f>
         <v>-</v>
       </c>
-      <c r="U29" s="4"/>
+      <c r="K29" s="118"/>
+      <c r="L29" s="118"/>
+      <c r="M29" s="118"/>
+      <c r="N29" s="118"/>
+      <c r="O29" s="118"/>
+      <c r="P29" s="118"/>
+      <c r="Q29" s="118"/>
+      <c r="R29" s="118"/>
+      <c r="S29" s="118"/>
+      <c r="T29" s="118"/>
+      <c r="U29" s="119"/>
     </row>
     <row r="30" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="10" t="str">
+      <c r="A30" s="5" t="str">
         <f t="shared" ref="A30:A39" si="10">IF(ISBLANK(A16),"",A16)</f>
         <v/>
       </c>
-      <c r="B30" s="7" t="str" cm="1">
+      <c r="B30" s="5" t="str" cm="1">
         <f t="array" ref="B30">IF(D16="", "", IF(AND(D16&lt;=MIN(K16:T16),E16&gt;=MAX(K16:T16)),"ACCEPT",IF(AND(K16:T16="OK"),"ACCEPT","REJECT")))</f>
         <v/>
       </c>
-      <c r="C30" s="7" t="str">
+      <c r="C30" s="5" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="D30" s="7" t="str">
+      <c r="D30" s="5" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="E30" s="7" t="str">
+      <c r="E30" s="5" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="F30" s="7">
+      <c r="F30" s="5">
         <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="G30" s="7">
+      <c r="G30" s="5">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="H30" s="7">
+      <c r="H30" s="5">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="I30" s="7">
+      <c r="I30" s="5">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J30" s="7" t="str">
+      <c r="J30" s="5" t="str">
         <f t="shared" si="9"/>
         <v>-</v>
       </c>
-      <c r="U30" s="4"/>
+      <c r="K30" s="118"/>
+      <c r="L30" s="118"/>
+      <c r="M30" s="118"/>
+      <c r="N30" s="118"/>
+      <c r="O30" s="118"/>
+      <c r="P30" s="118"/>
+      <c r="Q30" s="118"/>
+      <c r="R30" s="118"/>
+      <c r="S30" s="118"/>
+      <c r="T30" s="118"/>
+      <c r="U30" s="119"/>
     </row>
     <row r="31" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="10" t="str">
+      <c r="A31" s="5" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="B31" s="7" t="str" cm="1">
+      <c r="B31" s="5" t="str" cm="1">
         <f t="array" ref="B31">IF(D17="", "", IF(AND(D17&lt;=MIN(K17:T17),E17&gt;=MAX(K17:T17)),"ACCEPT",IF(AND(K17:T17="OK"),"ACCEPT","REJECT")))</f>
         <v/>
       </c>
-      <c r="C31" s="7" t="str">
+      <c r="C31" s="5" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="D31" s="7" t="str">
+      <c r="D31" s="5" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="E31" s="7" t="str">
+      <c r="E31" s="5" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="F31" s="7">
+      <c r="F31" s="5">
         <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="G31" s="7">
+      <c r="G31" s="5">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="H31" s="7">
+      <c r="H31" s="5">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="I31" s="7">
+      <c r="I31" s="5">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J31" s="7" t="str">
+      <c r="J31" s="5" t="str">
         <f t="shared" si="9"/>
         <v>-</v>
       </c>
-      <c r="U31" s="4"/>
+      <c r="K31" s="118"/>
+      <c r="L31" s="118"/>
+      <c r="M31" s="118"/>
+      <c r="N31" s="118"/>
+      <c r="O31" s="118"/>
+      <c r="P31" s="118"/>
+      <c r="Q31" s="118"/>
+      <c r="R31" s="118"/>
+      <c r="S31" s="118"/>
+      <c r="T31" s="118"/>
+      <c r="U31" s="119"/>
     </row>
     <row r="32" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="10" t="str">
+      <c r="A32" s="5" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="B32" s="7" t="str" cm="1">
+      <c r="B32" s="5" t="str" cm="1">
         <f t="array" ref="B32">IF(D18="", "", IF(AND(D18&lt;=MIN(K18:T18),E18&gt;=MAX(K18:T18)),"ACCEPT",IF(AND(K18:T18="OK"),"ACCEPT","REJECT")))</f>
         <v/>
       </c>
-      <c r="C32" s="7" t="str">
+      <c r="C32" s="5" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="D32" s="7" t="str">
+      <c r="D32" s="5" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="E32" s="7" t="str">
+      <c r="E32" s="5" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="F32" s="7">
+      <c r="F32" s="5">
         <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="G32" s="7">
+      <c r="G32" s="5">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="H32" s="7">
+      <c r="H32" s="5">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="I32" s="7">
+      <c r="I32" s="5">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J32" s="7" t="str">
+      <c r="J32" s="5" t="str">
         <f t="shared" si="9"/>
         <v>-</v>
       </c>
-      <c r="U32" s="4"/>
+      <c r="K32" s="118"/>
+      <c r="L32" s="118"/>
+      <c r="M32" s="118"/>
+      <c r="N32" s="118"/>
+      <c r="O32" s="118"/>
+      <c r="P32" s="118"/>
+      <c r="Q32" s="118"/>
+      <c r="R32" s="118"/>
+      <c r="S32" s="118"/>
+      <c r="T32" s="118"/>
+      <c r="U32" s="119"/>
     </row>
     <row r="33" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="10" t="str">
+      <c r="A33" s="5" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="B33" s="7" t="str" cm="1">
+      <c r="B33" s="5" t="str" cm="1">
         <f t="array" ref="B33">IF(D19="", "", IF(AND(D19&lt;=MIN(K19:T19),E19&gt;=MAX(K19:T19)),"ACCEPT",IF(AND(K19:T19="OK"),"ACCEPT","REJECT")))</f>
         <v/>
       </c>
-      <c r="C33" s="7" t="str">
+      <c r="C33" s="5" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="D33" s="7" t="str">
+      <c r="D33" s="5" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="E33" s="7" t="str">
+      <c r="E33" s="5" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="F33" s="7">
+      <c r="F33" s="5">
         <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="G33" s="7">
+      <c r="G33" s="5">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="H33" s="7">
+      <c r="H33" s="5">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="I33" s="7">
+      <c r="I33" s="5">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J33" s="7" t="str">
+      <c r="J33" s="5" t="str">
         <f t="shared" si="9"/>
         <v>-</v>
       </c>
-      <c r="U33" s="4"/>
+      <c r="K33" s="118"/>
+      <c r="L33" s="118"/>
+      <c r="M33" s="118"/>
+      <c r="N33" s="118"/>
+      <c r="O33" s="118"/>
+      <c r="P33" s="118"/>
+      <c r="Q33" s="118"/>
+      <c r="R33" s="118"/>
+      <c r="S33" s="118"/>
+      <c r="T33" s="118"/>
+      <c r="U33" s="119"/>
     </row>
     <row r="34" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="10" t="str">
+      <c r="A34" s="5" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="B34" s="7" t="str" cm="1">
+      <c r="B34" s="5" t="str" cm="1">
         <f t="array" ref="B34">IF(D20="", "", IF(AND(D20&lt;=MIN(K20:T20),E20&gt;=MAX(K20:T20)),"ACCEPT",IF(AND(K20:T20="OK"),"ACCEPT","REJECT")))</f>
         <v/>
       </c>
-      <c r="C34" s="7" t="str">
+      <c r="C34" s="5" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="D34" s="7" t="str">
+      <c r="D34" s="5" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="E34" s="7" t="str">
+      <c r="E34" s="5" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="F34" s="7">
+      <c r="F34" s="5">
         <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="G34" s="7">
+      <c r="G34" s="5">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="H34" s="7">
+      <c r="H34" s="5">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="I34" s="7">
+      <c r="I34" s="5">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J34" s="7" t="str">
+      <c r="J34" s="5" t="str">
         <f t="shared" si="9"/>
         <v>-</v>
       </c>
-      <c r="U34" s="4"/>
+      <c r="K34" s="118"/>
+      <c r="L34" s="118"/>
+      <c r="M34" s="118"/>
+      <c r="N34" s="118"/>
+      <c r="O34" s="118"/>
+      <c r="P34" s="118"/>
+      <c r="Q34" s="118"/>
+      <c r="R34" s="118"/>
+      <c r="S34" s="118"/>
+      <c r="T34" s="118"/>
+      <c r="U34" s="119"/>
     </row>
     <row r="35" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="10" t="str">
+      <c r="A35" s="5" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="B35" s="7" t="str" cm="1">
+      <c r="B35" s="5" t="str" cm="1">
         <f t="array" ref="B35">IF(D21="", "", IF(AND(D21&lt;=MIN(K21:T21),E21&gt;=MAX(K21:T21)),"ACCEPT",IF(AND(K21:T21="OK"),"ACCEPT","REJECT")))</f>
         <v/>
       </c>
-      <c r="C35" s="7" t="str">
+      <c r="C35" s="5" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="D35" s="7" t="str">
+      <c r="D35" s="5" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="E35" s="7" t="str">
+      <c r="E35" s="5" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="F35" s="7">
+      <c r="F35" s="5">
         <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="G35" s="7">
+      <c r="G35" s="5">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="H35" s="7">
+      <c r="H35" s="5">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="I35" s="7">
+      <c r="I35" s="5">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J35" s="7" t="str">
+      <c r="J35" s="5" t="str">
         <f t="shared" si="9"/>
         <v>-</v>
       </c>
-      <c r="U35" s="4"/>
+      <c r="K35" s="118"/>
+      <c r="L35" s="118"/>
+      <c r="M35" s="118"/>
+      <c r="N35" s="118"/>
+      <c r="O35" s="118"/>
+      <c r="P35" s="118"/>
+      <c r="Q35" s="118"/>
+      <c r="R35" s="118"/>
+      <c r="S35" s="118"/>
+      <c r="T35" s="118"/>
+      <c r="U35" s="119"/>
     </row>
     <row r="36" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="10" t="str">
+      <c r="A36" s="5" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="B36" s="7" t="str" cm="1">
+      <c r="B36" s="5" t="str" cm="1">
         <f t="array" ref="B36">IF(D22="", "", IF(AND(D22&lt;=MIN(K22:T22),E22&gt;=MAX(K22:T22)),"ACCEPT",IF(AND(K22:T22="OK"),"ACCEPT","REJECT")))</f>
         <v/>
       </c>
-      <c r="C36" s="7" t="str">
+      <c r="C36" s="5" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="D36" s="7" t="str">
+      <c r="D36" s="5" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="E36" s="7" t="str">
+      <c r="E36" s="5" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="F36" s="7">
+      <c r="F36" s="5">
         <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="G36" s="7">
+      <c r="G36" s="5">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="H36" s="7">
+      <c r="H36" s="5">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="I36" s="7">
+      <c r="I36" s="5">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J36" s="7" t="str">
+      <c r="J36" s="5" t="str">
         <f t="shared" si="9"/>
         <v>-</v>
       </c>
-      <c r="U36" s="4"/>
+      <c r="K36" s="118"/>
+      <c r="L36" s="118"/>
+      <c r="M36" s="118"/>
+      <c r="N36" s="118"/>
+      <c r="O36" s="118"/>
+      <c r="P36" s="118"/>
+      <c r="Q36" s="118"/>
+      <c r="R36" s="118"/>
+      <c r="S36" s="118"/>
+      <c r="T36" s="118"/>
+      <c r="U36" s="119"/>
     </row>
     <row r="37" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="10" t="str">
+      <c r="A37" s="5" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="B37" s="7" t="str" cm="1">
+      <c r="B37" s="5" t="str" cm="1">
         <f t="array" ref="B37">IF(D23="", "", IF(AND(D23&lt;=MIN(K23:T23),E23&gt;=MAX(K23:T23)),"ACCEPT",IF(AND(K23:T23="OK"),"ACCEPT","REJECT")))</f>
         <v/>
       </c>
-      <c r="C37" s="7" t="str">
+      <c r="C37" s="5" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="D37" s="7" t="str">
+      <c r="D37" s="5" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="E37" s="7" t="str">
+      <c r="E37" s="5" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="F37" s="7">
+      <c r="F37" s="5">
         <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="G37" s="7">
+      <c r="G37" s="5">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="H37" s="7">
+      <c r="H37" s="5">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="I37" s="7">
+      <c r="I37" s="5">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J37" s="7" t="str">
+      <c r="J37" s="5" t="str">
         <f t="shared" si="9"/>
         <v>-</v>
       </c>
-      <c r="U37" s="4"/>
+      <c r="K37" s="118"/>
+      <c r="L37" s="118"/>
+      <c r="M37" s="118"/>
+      <c r="N37" s="118"/>
+      <c r="O37" s="118"/>
+      <c r="P37" s="118"/>
+      <c r="Q37" s="118"/>
+      <c r="R37" s="118"/>
+      <c r="S37" s="118"/>
+      <c r="T37" s="118"/>
+      <c r="U37" s="119"/>
     </row>
     <row r="38" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="10" t="str">
+      <c r="A38" s="5" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="B38" s="7" t="str" cm="1">
+      <c r="B38" s="5" t="str" cm="1">
         <f t="array" ref="B38">IF(D24="", "", IF(AND(D24&lt;=MIN(K24:T24),E24&gt;=MAX(K24:T24)),"ACCEPT",IF(AND(K24:T24="OK"),"ACCEPT","REJECT")))</f>
         <v/>
       </c>
-      <c r="C38" s="7" t="str">
+      <c r="C38" s="5" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="D38" s="7" t="str">
+      <c r="D38" s="5" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="E38" s="7" t="str">
+      <c r="E38" s="5" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="F38" s="7">
+      <c r="F38" s="5">
         <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="G38" s="7">
+      <c r="G38" s="5">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="H38" s="7">
+      <c r="H38" s="5">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="I38" s="7">
+      <c r="I38" s="5">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J38" s="7" t="str">
+      <c r="J38" s="5" t="str">
         <f t="shared" si="9"/>
         <v>-</v>
       </c>
-      <c r="U38" s="4"/>
+      <c r="K38" s="118"/>
+      <c r="L38" s="118"/>
+      <c r="M38" s="118"/>
+      <c r="N38" s="118"/>
+      <c r="O38" s="118"/>
+      <c r="P38" s="118"/>
+      <c r="Q38" s="118"/>
+      <c r="R38" s="118"/>
+      <c r="S38" s="118"/>
+      <c r="T38" s="118"/>
+      <c r="U38" s="119"/>
     </row>
     <row r="39" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="10" t="str">
+      <c r="A39" s="5" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="B39" s="7" t="str" cm="1">
+      <c r="B39" s="5" t="str" cm="1">
         <f t="array" ref="B39">IF(D25="", "", IF(AND(D25&lt;=MIN(K25:T25),E25&gt;=MAX(K25:T25)),"ACCEPT",IF(AND(K25:T25="OK"),"ACCEPT","REJECT")))</f>
         <v/>
       </c>
-      <c r="C39" s="7" t="str">
+      <c r="C39" s="5" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="D39" s="7" t="str">
+      <c r="D39" s="5" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="E39" s="7" t="str">
+      <c r="E39" s="5" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="F39" s="7">
+      <c r="F39" s="5">
         <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="G39" s="7">
+      <c r="G39" s="5">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="H39" s="7">
+      <c r="H39" s="5">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="I39" s="7">
+      <c r="I39" s="5">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J39" s="7" t="str">
+      <c r="J39" s="5" t="str">
         <f t="shared" si="9"/>
         <v>-</v>
       </c>
-      <c r="U39" s="4"/>
+      <c r="K39" s="118"/>
+      <c r="L39" s="118"/>
+      <c r="M39" s="118"/>
+      <c r="N39" s="118"/>
+      <c r="O39" s="118"/>
+      <c r="P39" s="118"/>
+      <c r="Q39" s="118"/>
+      <c r="R39" s="118"/>
+      <c r="S39" s="118"/>
+      <c r="T39" s="118"/>
+      <c r="U39" s="119"/>
     </row>
     <row r="40" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="10" t="str">
+      <c r="A40" s="5" t="str">
         <f>IF(ISBLANK(A26),"",A26)</f>
         <v/>
       </c>
-      <c r="B40" s="7" t="str" cm="1">
+      <c r="B40" s="5" t="str" cm="1">
         <f t="array" ref="B40">IF(D26="", "", IF(AND(D26&lt;=MIN(K26:T26),E26&gt;=MAX(K26:T26)),"ACCEPT",IF(AND(K26:T26="OK"),"ACCEPT","REJECT")))</f>
         <v/>
       </c>
-      <c r="C40" s="7" t="str">
+      <c r="C40" s="5" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="D40" s="7" t="str">
+      <c r="D40" s="5" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="E40" s="7" t="str">
+      <c r="E40" s="5" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="F40" s="7">
+      <c r="F40" s="5">
         <f t="shared" si="5"/>
         <v>1</v>
       </c>
-      <c r="G40" s="7">
+      <c r="G40" s="5">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="H40" s="7">
+      <c r="H40" s="5">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="I40" s="7">
+      <c r="I40" s="5">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J40" s="7" t="str">
+      <c r="J40" s="5" t="str">
         <f t="shared" si="9"/>
         <v>-</v>
       </c>
-      <c r="U40" s="4"/>
+      <c r="K40" s="118"/>
+      <c r="L40" s="118"/>
+      <c r="M40" s="118"/>
+      <c r="N40" s="118"/>
+      <c r="O40" s="118"/>
+      <c r="P40" s="118"/>
+      <c r="Q40" s="118"/>
+      <c r="R40" s="118"/>
+      <c r="S40" s="118"/>
+      <c r="T40" s="118"/>
+      <c r="U40" s="119"/>
     </row>
     <row r="41" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="11"/>
-      <c r="B41" s="12"/>
-      <c r="C41" s="12"/>
-      <c r="D41" s="12"/>
-      <c r="E41" s="12"/>
-      <c r="U41" s="4"/>
+      <c r="A41" s="121"/>
+      <c r="B41" s="7"/>
+      <c r="C41" s="7"/>
+      <c r="D41" s="7"/>
+      <c r="E41" s="7"/>
+      <c r="F41" s="118"/>
+      <c r="G41" s="118"/>
+      <c r="H41" s="118"/>
+      <c r="I41" s="118"/>
+      <c r="J41" s="118"/>
+      <c r="K41" s="118"/>
+      <c r="L41" s="118"/>
+      <c r="M41" s="118"/>
+      <c r="N41" s="118"/>
+      <c r="O41" s="118"/>
+      <c r="P41" s="118"/>
+      <c r="Q41" s="118"/>
+      <c r="R41" s="118"/>
+      <c r="S41" s="118"/>
+      <c r="T41" s="118"/>
+      <c r="U41" s="119"/>
     </row>
     <row r="42" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="13" t="s">
+      <c r="A42" s="122" t="s">
         <v>15</v>
       </c>
-      <c r="B42" s="103"/>
-      <c r="C42" s="104"/>
-      <c r="D42" s="111" t="s">
+      <c r="B42" s="83"/>
+      <c r="C42" s="84"/>
+      <c r="D42" s="89" t="s">
         <v>17</v>
       </c>
-      <c r="E42" s="112"/>
-      <c r="G42" s="59" t="s">
+      <c r="E42" s="90"/>
+      <c r="F42" s="118"/>
+      <c r="G42" s="67" t="s">
         <v>57</v>
       </c>
-      <c r="H42" s="109"/>
-      <c r="I42" s="109"/>
-      <c r="J42" s="45"/>
-      <c r="L42" s="79" t="s">
+      <c r="H42" s="91"/>
+      <c r="I42" s="91"/>
+      <c r="J42" s="40"/>
+      <c r="K42" s="118"/>
+      <c r="L42" s="61" t="s">
         <v>58</v>
       </c>
-      <c r="M42" s="80"/>
-      <c r="N42" s="79" t="s">
+      <c r="M42" s="62"/>
+      <c r="N42" s="61" t="s">
         <v>4</v>
       </c>
-      <c r="O42" s="80"/>
-      <c r="Q42" s="79" t="s">
+      <c r="O42" s="62"/>
+      <c r="P42" s="118"/>
+      <c r="Q42" s="61" t="s">
         <v>58</v>
       </c>
-      <c r="R42" s="80"/>
-      <c r="S42" s="79" t="s">
+      <c r="R42" s="62"/>
+      <c r="S42" s="61" t="s">
         <v>4</v>
       </c>
-      <c r="T42" s="80"/>
-      <c r="U42" s="4"/>
+      <c r="T42" s="62"/>
+      <c r="U42" s="119"/>
     </row>
     <row r="43" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="5"/>
-      <c r="D43" s="113"/>
-      <c r="E43" s="114"/>
-      <c r="G43" s="65"/>
-      <c r="H43" s="110"/>
-      <c r="I43" s="110"/>
-      <c r="J43" s="49"/>
-      <c r="L43" s="44"/>
-      <c r="M43" s="45"/>
-      <c r="N43" s="44"/>
-      <c r="O43" s="45"/>
-      <c r="Q43" s="44"/>
-      <c r="R43" s="45"/>
-      <c r="S43" s="44"/>
-      <c r="T43" s="45"/>
-      <c r="U43" s="4"/>
+      <c r="A43" s="117"/>
+      <c r="B43" s="118"/>
+      <c r="C43" s="118"/>
+      <c r="D43" s="93"/>
+      <c r="E43" s="94"/>
+      <c r="F43" s="118"/>
+      <c r="G43" s="72"/>
+      <c r="H43" s="92"/>
+      <c r="I43" s="92"/>
+      <c r="J43" s="44"/>
+      <c r="K43" s="118"/>
+      <c r="L43" s="39"/>
+      <c r="M43" s="40"/>
+      <c r="N43" s="39"/>
+      <c r="O43" s="40"/>
+      <c r="P43" s="118"/>
+      <c r="Q43" s="39"/>
+      <c r="R43" s="40"/>
+      <c r="S43" s="39"/>
+      <c r="T43" s="40"/>
+      <c r="U43" s="119"/>
     </row>
     <row r="44" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="5" t="s">
+      <c r="A44" s="117" t="s">
         <v>16</v>
       </c>
-      <c r="B44" s="103"/>
-      <c r="C44" s="104"/>
-      <c r="D44" s="115"/>
-      <c r="E44" s="116"/>
-      <c r="G44" s="105" t="s">
+      <c r="B44" s="83"/>
+      <c r="C44" s="84"/>
+      <c r="D44" s="95"/>
+      <c r="E44" s="96"/>
+      <c r="F44" s="118"/>
+      <c r="G44" s="85" t="s">
         <v>68</v>
       </c>
-      <c r="H44" s="9" t="s">
+      <c r="H44" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="I44" s="108" t="s">
+      <c r="I44" s="88" t="s">
         <v>60</v>
       </c>
-      <c r="J44" s="108"/>
-      <c r="L44" s="46"/>
-      <c r="M44" s="47"/>
-      <c r="N44" s="46"/>
-      <c r="O44" s="47"/>
-      <c r="Q44" s="46"/>
-      <c r="R44" s="47"/>
-      <c r="S44" s="46"/>
-      <c r="T44" s="47"/>
-      <c r="U44" s="4"/>
+      <c r="J44" s="88"/>
+      <c r="K44" s="118"/>
+      <c r="L44" s="41"/>
+      <c r="M44" s="42"/>
+      <c r="N44" s="41"/>
+      <c r="O44" s="42"/>
+      <c r="P44" s="118"/>
+      <c r="Q44" s="41"/>
+      <c r="R44" s="42"/>
+      <c r="S44" s="41"/>
+      <c r="T44" s="42"/>
+      <c r="U44" s="119"/>
     </row>
     <row r="45" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="5"/>
-      <c r="D45" s="117"/>
-      <c r="E45" s="118"/>
-      <c r="G45" s="106"/>
-      <c r="H45" s="9" t="s">
+      <c r="A45" s="117"/>
+      <c r="B45" s="118"/>
+      <c r="C45" s="118"/>
+      <c r="D45" s="97"/>
+      <c r="E45" s="98"/>
+      <c r="F45" s="118"/>
+      <c r="G45" s="86"/>
+      <c r="H45" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="I45" s="108" t="s">
+      <c r="I45" s="88" t="s">
         <v>62</v>
       </c>
-      <c r="J45" s="108"/>
-      <c r="L45" s="48"/>
-      <c r="M45" s="49"/>
-      <c r="N45" s="48"/>
-      <c r="O45" s="49"/>
-      <c r="Q45" s="48"/>
-      <c r="R45" s="49"/>
-      <c r="S45" s="48"/>
-      <c r="T45" s="49"/>
-      <c r="U45" s="4"/>
+      <c r="J45" s="88"/>
+      <c r="K45" s="118"/>
+      <c r="L45" s="43"/>
+      <c r="M45" s="44"/>
+      <c r="N45" s="43"/>
+      <c r="O45" s="44"/>
+      <c r="P45" s="118"/>
+      <c r="Q45" s="43"/>
+      <c r="R45" s="44"/>
+      <c r="S45" s="43"/>
+      <c r="T45" s="44"/>
+      <c r="U45" s="119"/>
     </row>
     <row r="46" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="11"/>
-      <c r="B46" s="12"/>
-      <c r="C46" s="12"/>
-      <c r="D46" s="19" t="s">
+      <c r="A46" s="121"/>
+      <c r="B46" s="7"/>
+      <c r="C46" s="7"/>
+      <c r="D46" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="E46" s="14"/>
-      <c r="G46" s="107"/>
-      <c r="H46" s="9" t="s">
+      <c r="E46" s="8"/>
+      <c r="F46" s="118"/>
+      <c r="G46" s="87"/>
+      <c r="H46" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="I46" s="108" t="s">
+      <c r="I46" s="88" t="s">
         <v>64</v>
       </c>
-      <c r="J46" s="108"/>
-      <c r="L46" s="25" t="s">
+      <c r="J46" s="88"/>
+      <c r="K46" s="118"/>
+      <c r="L46" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="M46" s="6"/>
-      <c r="N46" s="25" t="s">
+      <c r="M46" s="4"/>
+      <c r="N46" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="O46" s="6"/>
-      <c r="Q46" s="25" t="s">
+      <c r="O46" s="4"/>
+      <c r="P46" s="118"/>
+      <c r="Q46" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="R46" s="6"/>
-      <c r="S46" s="25" t="s">
+      <c r="R46" s="4"/>
+      <c r="S46" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="T46" s="6"/>
-      <c r="U46" s="4"/>
+      <c r="T46" s="4"/>
+      <c r="U46" s="119"/>
     </row>
     <row r="47" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="11"/>
-      <c r="B47" s="12"/>
-      <c r="C47" s="12"/>
-      <c r="D47" s="12"/>
-      <c r="E47" s="12"/>
-      <c r="F47" s="12"/>
-      <c r="G47" s="12"/>
-      <c r="H47" s="12"/>
-      <c r="I47" s="12"/>
-      <c r="J47" s="12"/>
-      <c r="K47" s="12"/>
-      <c r="L47" s="12"/>
-      <c r="M47" s="12"/>
-      <c r="N47" s="12"/>
-      <c r="O47" s="12"/>
-      <c r="P47" s="12"/>
-      <c r="Q47" s="12"/>
-      <c r="R47" s="12"/>
-      <c r="S47" s="12"/>
-      <c r="T47" s="12"/>
-      <c r="U47" s="15"/>
-    </row>
-    <row r="48" spans="1:21" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="16"/>
-      <c r="B48" s="17"/>
-      <c r="C48" s="17"/>
-      <c r="D48" s="17"/>
-      <c r="E48" s="17"/>
-      <c r="F48" s="17"/>
-      <c r="G48" s="17"/>
-      <c r="H48" s="17"/>
-      <c r="I48" s="17"/>
-      <c r="J48" s="17"/>
-      <c r="K48" s="17"/>
-      <c r="L48" s="75" t="s">
+      <c r="A47" s="121"/>
+      <c r="B47" s="7"/>
+      <c r="C47" s="7"/>
+      <c r="D47" s="7"/>
+      <c r="E47" s="7"/>
+      <c r="F47" s="7"/>
+      <c r="G47" s="7"/>
+      <c r="H47" s="7"/>
+      <c r="I47" s="7"/>
+      <c r="J47" s="7"/>
+      <c r="K47" s="7"/>
+      <c r="L47" s="7"/>
+      <c r="M47" s="7"/>
+      <c r="N47" s="7"/>
+      <c r="O47" s="7"/>
+      <c r="P47" s="7"/>
+      <c r="Q47" s="7"/>
+      <c r="R47" s="7"/>
+      <c r="S47" s="7"/>
+      <c r="T47" s="7"/>
+      <c r="U47" s="123"/>
+    </row>
+    <row r="48" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="121"/>
+      <c r="B48" s="7"/>
+      <c r="C48" s="7"/>
+      <c r="D48" s="7"/>
+      <c r="E48" s="7"/>
+      <c r="F48" s="7"/>
+      <c r="G48" s="7"/>
+      <c r="H48" s="7"/>
+      <c r="I48" s="7"/>
+      <c r="J48" s="7"/>
+      <c r="K48" s="7"/>
+      <c r="L48" s="82" t="s">
         <v>67</v>
       </c>
-      <c r="M48" s="75"/>
-      <c r="N48" s="75"/>
-      <c r="O48" s="76" t="s">
+      <c r="M48" s="82"/>
+      <c r="N48" s="82"/>
+      <c r="O48" s="124" t="s">
         <v>66</v>
       </c>
-      <c r="P48" s="76"/>
-      <c r="Q48" s="76"/>
-      <c r="R48" s="76"/>
-      <c r="S48" s="76" t="s">
+      <c r="P48" s="124"/>
+      <c r="Q48" s="124"/>
+      <c r="R48" s="124"/>
+      <c r="S48" s="124" t="s">
         <v>65</v>
       </c>
-      <c r="T48" s="76"/>
-      <c r="U48" s="77"/>
+      <c r="T48" s="124"/>
+      <c r="U48" s="125"/>
     </row>
     <row r="49" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="50" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -3839,58 +3762,24 @@
     <protectedRange algorithmName="SHA-512" hashValue="e8n0DY2l0+gBcmtbdmdOldou2feyh808cNYkqqQvqM4Cxw3lge815bmlq59VAVuRm9kfLOFkgitWSyXhyj/Q5Q==" saltValue="kF6gufaZSgPuxk6T2iYUWA==" spinCount="100000" sqref="L9 J9 P9 I6 K6 M6 O6 S7" name="WORKINSTRUCTION_EDITRANGE"/>
     <protectedRange algorithmName="SHA-512" hashValue="YrFhROLDD5jOGTRCiqJ4P5er6/CR5vEaYX7Pzp+9fY7EmPEASJhfIv1Ui3ockLk1g4gNGdmazNbyESfxKzE7hQ==" saltValue="mudhKlzvxzTwFuCj6VIXiA==" spinCount="100000" sqref="S8 A15:F26 S4:U6" name="BUYOFF_EDITRANGE"/>
   </protectedRanges>
-  <mergeCells count="94">
-    <mergeCell ref="Q4:R5"/>
-    <mergeCell ref="S4:U4"/>
-    <mergeCell ref="S5:U5"/>
-    <mergeCell ref="Q6:R6"/>
-    <mergeCell ref="Q7:R7"/>
-    <mergeCell ref="O9:P9"/>
-    <mergeCell ref="I13:J14"/>
-    <mergeCell ref="K13:O13"/>
-    <mergeCell ref="P13:T13"/>
-    <mergeCell ref="Q43:R45"/>
-    <mergeCell ref="S43:T45"/>
-    <mergeCell ref="S48:U48"/>
-    <mergeCell ref="O48:R48"/>
-    <mergeCell ref="L48:N48"/>
-    <mergeCell ref="Q8:R8"/>
-    <mergeCell ref="K1:R3"/>
-    <mergeCell ref="S1:U3"/>
-    <mergeCell ref="A1:B3"/>
-    <mergeCell ref="C1:J3"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="K4:M4"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="S7:U7"/>
-    <mergeCell ref="S6:U6"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="K5:M5"/>
-    <mergeCell ref="N5:P5"/>
-    <mergeCell ref="H6:J8"/>
-    <mergeCell ref="K6:M8"/>
-    <mergeCell ref="N6:P8"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="C5:G5"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="Q11:R11"/>
-    <mergeCell ref="G10:G11"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="N10:N11"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="B13:C14"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="I17:J17"/>
+  <mergeCells count="97">
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="G44:G46"/>
+    <mergeCell ref="I44:J44"/>
+    <mergeCell ref="I45:J45"/>
+    <mergeCell ref="I46:J46"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="H42:J43"/>
+    <mergeCell ref="D43:E45"/>
+    <mergeCell ref="G42:G43"/>
+    <mergeCell ref="I26:J26"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="I18:J18"/>
     <mergeCell ref="A27:J27"/>
@@ -3907,33 +3796,70 @@
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="I19:J19"/>
     <mergeCell ref="B23:C23"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="G44:G46"/>
-    <mergeCell ref="I44:J44"/>
-    <mergeCell ref="I45:J45"/>
-    <mergeCell ref="I46:J46"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="H42:J43"/>
-    <mergeCell ref="D43:E45"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="G10:G11"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="N10:N11"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="B13:C14"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="C5:G5"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="N5:P5"/>
+    <mergeCell ref="H6:J8"/>
+    <mergeCell ref="K6:M8"/>
+    <mergeCell ref="N6:P8"/>
+    <mergeCell ref="A1:B3"/>
+    <mergeCell ref="C1:J3"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="K4:M4"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="S48:U48"/>
+    <mergeCell ref="O48:R48"/>
+    <mergeCell ref="L48:N48"/>
+    <mergeCell ref="Q8:R8"/>
+    <mergeCell ref="K1:R3"/>
+    <mergeCell ref="S1:U3"/>
+    <mergeCell ref="S7:U7"/>
+    <mergeCell ref="S6:U6"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="Q11:R11"/>
     <mergeCell ref="L43:M45"/>
     <mergeCell ref="N43:O45"/>
     <mergeCell ref="S42:T42"/>
-    <mergeCell ref="G42:G43"/>
     <mergeCell ref="L42:M42"/>
     <mergeCell ref="N42:O42"/>
     <mergeCell ref="Q42:R42"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="O9:P9"/>
+    <mergeCell ref="I13:J14"/>
+    <mergeCell ref="K13:O13"/>
+    <mergeCell ref="P13:T13"/>
+    <mergeCell ref="Q43:R45"/>
+    <mergeCell ref="S43:T45"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="Q10:R10"/>
+    <mergeCell ref="S10:U10"/>
+    <mergeCell ref="S11:U11"/>
+    <mergeCell ref="Q4:R5"/>
+    <mergeCell ref="S4:U4"/>
+    <mergeCell ref="S5:U5"/>
+    <mergeCell ref="Q6:R6"/>
+    <mergeCell ref="Q7:R7"/>
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <conditionalFormatting sqref="B29:B40">
@@ -3944,7 +3870,7 @@
       <formula>"ACCEPT"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F15:F26" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"-,QC,QCF"</formula1>
     </dataValidation>

</xml_diff>